<commit_message>
Update template – add conditional formatting for account currency
</commit_message>
<xml_diff>
--- a/finview_transactions_template.xlsx
+++ b/finview_transactions_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pxheller/Development/finview/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBA796FF-CEC9-D542-A84E-793E89919CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E20E486-081B-4349-877E-0AC61F1F858A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="800" windowWidth="35200" windowHeight="22580" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10580" yWindow="800" windowWidth="24620" windowHeight="22580" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" state="hidden" r:id="rId1"/>
@@ -197,18 +197,30 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="9">
     <dxf>
-      <numFmt numFmtId="166" formatCode="_([$CHF]\ * #,##0.00_);_([$CHF]\ * \(#,##0.00\);_([$CHF]\ * &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="167" formatCode="_([$GBP]\ * #,##0.00_);_([$GBP]\ * \(#,##0.00\);_([$GBP]\ * &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="_([$GBP]\ * #,##0.00_);_([$GBP]\ * \(#,##0.00\);_([$GBP]\ * &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="169" formatCode="_([$USD]\ * #,##0.00_);_([$USD]\ * \(#,##0.00\);_([$USD]\ * &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="168" formatCode="_([$EUR]\ * #,##0.00_);_([$EUR]\ * \(#,##0.00\);_([$EUR]\ * &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="167" formatCode="_([$USD]\ * #,##0.00_);_([$USD]\ * \(#,##0.00\);_([$USD]\ * &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="166" formatCode="_([$CHF]\ * #,##0.00_);_([$CHF]\ * \(#,##0.00\);_([$CHF]\ * &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="_([$CHF]\ * #,##0.00_);_([$CHF]\ * \(#,##0.00\);_([$CHF]\ * &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="_([$GBP]\ * #,##0.00_);_([$GBP]\ * \(#,##0.00\);_([$GBP]\ * &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="_([$EUR]\ * #,##0.00_);_([$EUR]\ * \(#,##0.00\);_([$EUR]\ * &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="169" formatCode="_([$USD]\ * #,##0.00_);_([$USD]\ * \(#,##0.00\);_([$USD]\ * &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="ddd* mmm\ d\,\ yyyy\ h:mm\ AM/PM"/>
@@ -261,7 +273,7 @@
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="original_value"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="original_currency"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="value_in_account_currency"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="date" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="date" dataDxfId="8"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="category"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="category_id"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="reviewed"/>
@@ -700,9 +712,9 @@
     <col min="3" max="3" width="13" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="18.33203125" customWidth="1"/>
     <col min="5" max="5" width="36" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" customWidth="1"/>
-    <col min="7" max="7" width="9" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="25.33203125" customWidth="1"/>
+    <col min="6" max="6" width="25.83203125" customWidth="1"/>
+    <col min="7" max="7" width="3.83203125" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="25.83203125" customWidth="1"/>
     <col min="9" max="9" width="21.5" customWidth="1"/>
     <col min="10" max="10" width="20.6640625" customWidth="1"/>
     <col min="11" max="11" width="13.33203125" hidden="1" customWidth="1"/>
@@ -804,16 +816,16 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <conditionalFormatting sqref="F6">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="7" priority="5">
       <formula>G6="USD"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="6" priority="6">
       <formula>G6="EUR"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="7" stopIfTrue="1">
       <formula>G6="GBP"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="4" priority="8">
       <formula>G6="CHF"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -828,6 +840,37 @@
     <tablePart r:id="rId1"/>
   </tableParts>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="expression" priority="4" id="{99DDDF38-905A-E64F-8ED5-A9DA353C1078}">
+            <xm:f>_xlfn.XLOOKUP(C6,Accounts!A2:A2000,Accounts!C2:C2000)="CHF"</xm:f>
+            <x14:dxf>
+              <numFmt numFmtId="166" formatCode="_([$CHF]\ * #,##0.00_);_([$CHF]\ * \(#,##0.00\);_([$CHF]\ * &quot;-&quot;??_);_(@_)"/>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="expression" priority="3" id="{88D74382-B62E-6746-80F1-B80C5FFB9290}">
+            <xm:f>_xlfn.XLOOKUP(C6,Accounts!A2:A2000,Accounts!C2:C2000)="GBP"</xm:f>
+            <x14:dxf>
+              <numFmt numFmtId="167" formatCode="_([$GBP]\ * #,##0.00_);_([$GBP]\ * \(#,##0.00\);_([$GBP]\ * &quot;-&quot;??_);_(@_)"/>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="expression" priority="2" id="{ED1A46FA-080F-5048-8DA0-86D3F7F57ECE}">
+            <xm:f>_xlfn.XLOOKUP(C6,Accounts!A2:A2000,Accounts!C2:C2000)="USD"</xm:f>
+            <x14:dxf>
+              <numFmt numFmtId="169" formatCode="_([$USD]\ * #,##0.00_);_([$USD]\ * \(#,##0.00\);_([$USD]\ * &quot;-&quot;??_);_(@_)"/>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="expression" priority="1" id="{1869173A-BE23-7A43-AB4E-001888C14FC9}">
+            <xm:f>_xlfn.XLOOKUP(C6,Accounts!A2:A2000,Accounts!C2:C2000)="EUR"</xm:f>
+            <x14:dxf>
+              <numFmt numFmtId="168" formatCode="_([$EUR]\ * #,##0.00_);_([$EUR]\ * \(#,##0.00\);_([$EUR]\ * &quot;-&quot;??_);_(@_)"/>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>H6</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" errorTitle="Invalid Category" error="Please select a valid category" xr:uid="{00000000-0002-0000-0200-000000000000}">

</xml_diff>